<commit_message>
Update agent metadata and customer list export
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/exports/customer-list.xlsx
+++ b/exports/customer-list.xlsx
@@ -90,13 +90,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="61" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="62" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,18 +425,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H82"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="36.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="25.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" t="str">
         <v>Customer Name</v>
       </c>
@@ -476,20 +462,20 @@
       <c r="C2" t="str">
         <v>sales@3peaksbranding.co.uk</v>
       </c>
-      <c r="D2" s="1" t="str">
+      <c r="D2" t="str">
         <v>07973 627364</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2">
         <v>52</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2">
         <v>19.7</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2">
         <v>2.02</v>
       </c>
-      <c r="H2" s="5" t="d">
-        <v>2026-09-16T00:00:00.000Z</v>
+      <c r="H2" s="1" t="str">
+        <v>16/09/2026</v>
       </c>
     </row>
     <row r="3">
@@ -502,10 +488,10 @@
       <c r="C3" t="str">
         <v>forty1prints@outlook.com</v>
       </c>
-      <c r="D3" s="1" t="str">
+      <c r="D3" t="str">
         <v/>
       </c>
-      <c r="E3" s="2">
+      <c r="E3">
         <v>0</v>
       </c>
     </row>
@@ -519,20 +505,20 @@
       <c r="C4" t="str">
         <v>accounts@absolutepromotions.co.uk</v>
       </c>
-      <c r="D4" s="1" t="str">
+      <c r="D4" t="str">
         <v>01892 513361</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4">
         <v>2</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4">
         <v>273.5</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4">
         <v>1.43</v>
       </c>
-      <c r="H4" s="5" t="d">
-        <v>2026-08-06T00:00:00.000Z</v>
+      <c r="H4" s="1" t="str">
+        <v>06/08/2026</v>
       </c>
     </row>
     <row r="5">
@@ -545,20 +531,20 @@
       <c r="C5" t="str">
         <v>trophies@affinitypromotionsandevents.co.uk</v>
       </c>
-      <c r="D5" s="1" t="str">
+      <c r="D5" t="str">
         <v/>
       </c>
-      <c r="E5" s="2">
+      <c r="E5">
         <v>7</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5">
         <v>240.7</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5">
         <v>3.37</v>
       </c>
-      <c r="H5" s="5" t="d">
-        <v>2026-03-29T00:00:00.000Z</v>
+      <c r="H5" s="1" t="str">
+        <v>29/03/2026</v>
       </c>
     </row>
     <row r="6">
@@ -571,20 +557,20 @@
       <c r="C6" t="str">
         <v>geoff@ambitionsport.com</v>
       </c>
-      <c r="D6" s="1" t="str">
+      <c r="D6" t="str">
         <v>07773 773027</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6">
         <v>4</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6">
         <v>74.5</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6">
         <v>1.71</v>
       </c>
-      <c r="H6" s="5" t="d">
-        <v>2026-09-16T00:00:00.000Z</v>
+      <c r="H6" s="1" t="str">
+        <v>16/09/2026</v>
       </c>
     </row>
     <row r="7">
@@ -597,20 +583,20 @@
       <c r="C7" t="str">
         <v>johnw@artisanshirts.co.uk</v>
       </c>
-      <c r="D7" s="1" t="str">
+      <c r="D7" t="str">
         <v>01865 820400</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7">
         <v>1</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7">
         <v>1255</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7">
         <v>1.31</v>
       </c>
-      <c r="H7" s="5" t="d">
-        <v>2026-07-09T00:00:00.000Z</v>
+      <c r="H7" s="1" t="str">
+        <v>09/07/2026</v>
       </c>
     </row>
     <row r="8">
@@ -623,17 +609,17 @@
       <c r="C8" t="str">
         <v>sales@ascotpromotions.co.uk</v>
       </c>
-      <c r="D8" s="1" t="str">
+      <c r="D8" t="str">
         <v>01344893263</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8">
         <v>2</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8">
         <v>61.5</v>
       </c>
-      <c r="H8" s="5" t="d">
-        <v>2025-12-03T00:00:00.000Z</v>
+      <c r="H8" s="1" t="str">
+        <v>03/12/2025</v>
       </c>
     </row>
     <row r="9">
@@ -646,17 +632,17 @@
       <c r="C9" t="str">
         <v>david.wilton@corporateclothingwear.com</v>
       </c>
-      <c r="D9" s="1" t="str">
+      <c r="D9" t="str">
         <v/>
       </c>
-      <c r="E9" s="2">
+      <c r="E9">
         <v>10</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9">
         <v>33.5</v>
       </c>
-      <c r="H9" s="5" t="d">
-        <v>2025-11-05T00:00:00.000Z</v>
+      <c r="H9" s="1" t="str">
+        <v>05/11/2025</v>
       </c>
     </row>
     <row r="10">
@@ -669,20 +655,20 @@
       <c r="C10" t="str">
         <v>info@b46group.co.uk</v>
       </c>
-      <c r="D10" s="1" t="str">
+      <c r="D10" t="str">
         <v>07814640522</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10">
         <v>4</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10">
         <v>13.3</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10">
         <v>2.65</v>
       </c>
-      <c r="H10" s="5" t="d">
-        <v>2026-02-17T00:00:00.000Z</v>
+      <c r="H10" s="1" t="str">
+        <v>17/02/2026</v>
       </c>
     </row>
     <row r="11">
@@ -695,20 +681,20 @@
       <c r="C11" t="str">
         <v>info@belgravepm.co.uk</v>
       </c>
-      <c r="D11" s="1" t="str">
+      <c r="D11" t="str">
         <v>01615053219</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11">
         <v>19</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11">
         <v>11.1</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11">
         <v>2.67</v>
       </c>
-      <c r="H11" s="5" t="d">
-        <v>2026-09-16T00:00:00.000Z</v>
+      <c r="H11" s="1" t="str">
+        <v>16/09/2026</v>
       </c>
     </row>
     <row r="12">
@@ -721,20 +707,20 @@
       <c r="C12" t="str">
         <v>graphics@brtgroup.co.uk</v>
       </c>
-      <c r="D12" s="1" t="str">
+      <c r="D12" t="str">
         <v>01527400092</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12">
         <v>16</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12">
         <v>67.9</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12">
         <v>1.55</v>
       </c>
-      <c r="H12" s="5" t="d">
-        <v>2026-09-08T00:00:00.000Z</v>
+      <c r="H12" s="1" t="str">
+        <v>08/09/2026</v>
       </c>
     </row>
     <row r="13">
@@ -747,20 +733,20 @@
       <c r="C13" t="str">
         <v>hello@bangonbranding.co.uk</v>
       </c>
-      <c r="D13" s="1" t="str">
+      <c r="D13" t="str">
         <v>02392800688</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13">
         <v>5</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13">
         <v>93</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13">
         <v>2.59</v>
       </c>
-      <c r="H13" s="5" t="d">
-        <v>2026-09-15T00:00:00.000Z</v>
+      <c r="H13" s="1" t="str">
+        <v>15/09/2026</v>
       </c>
     </row>
     <row r="14">
@@ -773,20 +759,20 @@
       <c r="C14" t="str">
         <v>saadmansoor1020@gmail.com</v>
       </c>
-      <c r="D14" s="1" t="str">
+      <c r="D14" t="str">
         <v/>
       </c>
-      <c r="E14" s="2">
+      <c r="E14">
         <v>22</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14">
         <v>37.5</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14">
         <v>3.05</v>
       </c>
-      <c r="H14" s="5" t="d">
-        <v>2026-09-01T00:00:00.000Z</v>
+      <c r="H14" s="1" t="str">
+        <v>01/09/2026</v>
       </c>
     </row>
     <row r="15">
@@ -799,10 +785,10 @@
       <c r="C15" t="str">
         <v>michaelstanley@brandableclothing.co.uk</v>
       </c>
-      <c r="D15" s="1" t="str">
+      <c r="D15" t="str">
         <v>03030033630</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15">
         <v>0</v>
       </c>
     </row>
@@ -816,20 +802,20 @@
       <c r="C16" t="str">
         <v>ranjit@brandinginc.co.uk</v>
       </c>
-      <c r="D16" s="1" t="str">
+      <c r="D16" t="str">
         <v>07926432883</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16">
         <v>79</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16">
         <v>37.5</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16">
         <v>1.59</v>
       </c>
-      <c r="H16" s="5" t="d">
-        <v>2026-07-28T00:00:00.000Z</v>
+      <c r="H16" s="1" t="str">
+        <v>28/07/2026</v>
       </c>
     </row>
     <row r="17">
@@ -842,10 +828,10 @@
       <c r="C17" t="str">
         <v>contact@brosweyth.co.uk</v>
       </c>
-      <c r="D17" s="1" t="str">
+      <c r="D17" t="str">
         <v>07500895700</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17">
         <v>0</v>
       </c>
     </row>
@@ -859,20 +845,20 @@
       <c r="C18" t="str">
         <v>everton@creativeco.co.uk</v>
       </c>
-      <c r="D18" s="1" t="str">
+      <c r="D18" t="str">
         <v>07931381275</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18">
         <v>1</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18">
         <v>4</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18">
         <v>2.17</v>
       </c>
-      <c r="H18" s="5" t="d">
-        <v>2026-02-20T00:00:00.000Z</v>
+      <c r="H18" s="1" t="str">
+        <v>20/02/2026</v>
       </c>
     </row>
     <row r="19">
@@ -885,10 +871,10 @@
       <c r="C19" t="str">
         <v>bob@conceptpm.com</v>
       </c>
-      <c r="D19" s="1" t="str">
+      <c r="D19" t="str">
         <v>07950255208</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19">
         <v>0</v>
       </c>
     </row>
@@ -902,20 +888,20 @@
       <c r="C20" t="str">
         <v>Creations-4-you@hotmail.com</v>
       </c>
-      <c r="D20" s="1" t="str">
+      <c r="D20" t="str">
         <v/>
       </c>
-      <c r="E20" s="2">
+      <c r="E20">
         <v>3</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20">
         <v>5.7</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20">
         <v>3.29</v>
       </c>
-      <c r="H20" s="5" t="d">
-        <v>2026-07-08T00:00:00.000Z</v>
+      <c r="H20" s="1" t="str">
+        <v>08/07/2026</v>
       </c>
     </row>
     <row r="21">
@@ -928,20 +914,20 @@
       <c r="C21" t="str">
         <v>tracy@creative-embroiders.co.uk</v>
       </c>
-      <c r="D21" s="1" t="str">
+      <c r="D21" t="str">
         <v/>
       </c>
-      <c r="E21" s="2">
+      <c r="E21">
         <v>1</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21">
         <v>101</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21">
         <v>1.52</v>
       </c>
-      <c r="H21" s="5" t="d">
-        <v>2026-02-11T00:00:00.000Z</v>
+      <c r="H21" s="1" t="str">
+        <v>11/02/2026</v>
       </c>
     </row>
     <row r="22">
@@ -954,20 +940,20 @@
       <c r="C22" t="str">
         <v>curvyrails@gmail.com</v>
       </c>
-      <c r="D22" s="1" t="str">
+      <c r="D22" t="str">
         <v>07301080811</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22">
         <v>2</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22">
         <v>72</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22">
         <v>1.9</v>
       </c>
-      <c r="H22" s="5" t="d">
-        <v>2026-09-13T00:00:00.000Z</v>
+      <c r="H22" s="1" t="str">
+        <v>13/09/2026</v>
       </c>
     </row>
     <row r="23">
@@ -980,20 +966,20 @@
       <c r="C23" t="str">
         <v>customisedprints3@yahoo.com</v>
       </c>
-      <c r="D23" s="1" t="str">
+      <c r="D23" t="str">
         <v>028 7776 7783</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23">
         <v>12</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23">
         <v>112.3</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23">
         <v>1.66</v>
       </c>
-      <c r="H23" s="5" t="d">
-        <v>2026-08-03T00:00:00.000Z</v>
+      <c r="H23" s="1" t="str">
+        <v>03/08/2026</v>
       </c>
     </row>
     <row r="24">
@@ -1006,17 +992,17 @@
       <c r="C24" t="str">
         <v>forrest.druhbelts@gmail.com</v>
       </c>
-      <c r="D24" s="1" t="str">
+      <c r="D24" t="str">
         <v>07557379622</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24">
         <v>1</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24">
         <v>10</v>
       </c>
-      <c r="H24" s="5" t="d">
-        <v>2026-01-06T00:00:00.000Z</v>
+      <c r="H24" s="1" t="str">
+        <v>06/01/2026</v>
       </c>
     </row>
     <row r="25">
@@ -1029,17 +1015,17 @@
       <c r="C25" t="str">
         <v>darrel@eastpointsports.net</v>
       </c>
-      <c r="D25" s="1" t="str">
+      <c r="D25" t="str">
         <v/>
       </c>
-      <c r="E25" s="2">
+      <c r="E25">
         <v>3</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25">
         <v>10</v>
       </c>
-      <c r="H25" s="5" t="d">
-        <v>2025-11-13T00:00:00.000Z</v>
+      <c r="H25" s="1" t="str">
+        <v>13/11/2025</v>
       </c>
     </row>
     <row r="26">
@@ -1052,20 +1038,20 @@
       <c r="C26" t="str">
         <v>hello@eastyorkshireworkwear.co.uk</v>
       </c>
-      <c r="D26" s="1" t="str">
+      <c r="D26" t="str">
         <v>07989556587</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26">
         <v>75</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F26">
         <v>34.9</v>
       </c>
-      <c r="G26" s="4">
+      <c r="G26">
         <v>1.69</v>
       </c>
-      <c r="H26" s="5" t="d">
-        <v>2026-08-31T00:00:00.000Z</v>
+      <c r="H26" s="1" t="str">
+        <v>31/08/2026</v>
       </c>
     </row>
     <row r="27">
@@ -1078,20 +1064,20 @@
       <c r="C27" t="str">
         <v>sales@embroideryloft.co.uk</v>
       </c>
-      <c r="D27" s="1" t="str">
+      <c r="D27" t="str">
         <v>01293 863915</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27">
         <v>1</v>
       </c>
-      <c r="F27" s="3">
+      <c r="F27">
         <v>21</v>
       </c>
-      <c r="G27" s="4">
+      <c r="G27">
         <v>2.26</v>
       </c>
-      <c r="H27" s="5" t="d">
-        <v>2026-08-27T00:00:00.000Z</v>
+      <c r="H27" s="1" t="str">
+        <v>27/08/2026</v>
       </c>
     </row>
     <row r="28">
@@ -1104,20 +1090,20 @@
       <c r="C28" t="str">
         <v>info@harrogateembroidery.com</v>
       </c>
-      <c r="D28" s="1" t="str">
+      <c r="D28" t="str">
         <v>07500 861192</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28">
         <v>4</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28">
         <v>24.5</v>
       </c>
-      <c r="G28" s="4">
+      <c r="G28">
         <v>3.29</v>
       </c>
-      <c r="H28" s="5" t="d">
-        <v>2026-09-18T00:00:00.000Z</v>
+      <c r="H28" s="1" t="str">
+        <v>18/09/2026</v>
       </c>
     </row>
     <row r="29">
@@ -1130,20 +1116,20 @@
       <c r="C29" t="str">
         <v>sales@hartlandhoodies.com</v>
       </c>
-      <c r="D29" s="1" t="str">
+      <c r="D29" t="str">
         <v>07771703247</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29">
         <v>7</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F29">
         <v>7.4</v>
       </c>
-      <c r="G29" s="4">
+      <c r="G29">
         <v>2.77</v>
       </c>
-      <c r="H29" s="5" t="d">
-        <v>2026-02-13T00:00:00.000Z</v>
+      <c r="H29" s="1" t="str">
+        <v>13/02/2026</v>
       </c>
     </row>
     <row r="30">
@@ -1156,10 +1142,10 @@
       <c r="C30" t="str">
         <v>claire@embroidery.london</v>
       </c>
-      <c r="D30" s="1" t="str">
+      <c r="D30" t="str">
         <v/>
       </c>
-      <c r="E30" s="2">
+      <c r="E30">
         <v>0</v>
       </c>
     </row>
@@ -1173,17 +1159,17 @@
       <c r="C31" t="str">
         <v>sales@hazzad.golf</v>
       </c>
-      <c r="D31" s="1" t="str">
+      <c r="D31" t="str">
         <v/>
       </c>
-      <c r="E31" s="2">
+      <c r="E31">
         <v>1</v>
       </c>
-      <c r="F31" s="3">
+      <c r="F31">
         <v>10</v>
       </c>
-      <c r="H31" s="5" t="d">
-        <v>2026-01-23T00:00:00.000Z</v>
+      <c r="H31" s="1" t="str">
+        <v>23/01/2026</v>
       </c>
     </row>
     <row r="32">
@@ -1196,20 +1182,20 @@
       <c r="C32" t="str">
         <v>info@iddancewear.com</v>
       </c>
-      <c r="D32" s="1" t="str">
+      <c r="D32" t="str">
         <v>07706799817</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32">
         <v>19</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32">
         <v>46</v>
       </c>
-      <c r="G32" s="4">
+      <c r="G32">
         <v>2.19</v>
       </c>
-      <c r="H32" s="5" t="d">
-        <v>2026-07-26T00:00:00.000Z</v>
+      <c r="H32" s="1" t="str">
+        <v>26/07/2026</v>
       </c>
     </row>
     <row r="33">
@@ -1222,20 +1208,20 @@
       <c r="C33" t="str">
         <v>tony@intersafety.co.uk</v>
       </c>
-      <c r="D33" s="1" t="str">
+      <c r="D33" t="str">
         <v>07919199075</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33">
         <v>11</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33">
         <v>643.8</v>
       </c>
-      <c r="G33" s="4">
+      <c r="G33">
         <v>1.19</v>
       </c>
-      <c r="H33" s="5" t="d">
-        <v>2026-09-14T00:00:00.000Z</v>
+      <c r="H33" s="1" t="str">
+        <v>14/09/2026</v>
       </c>
     </row>
     <row r="34">
@@ -1248,10 +1234,10 @@
       <c r="C34" t="str">
         <v>info@jeembroidery.com</v>
       </c>
-      <c r="D34" s="1" t="str">
+      <c r="D34" t="str">
         <v>01524 748348</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34">
         <v>0</v>
       </c>
     </row>
@@ -1265,20 +1251,20 @@
       <c r="C35" t="str">
         <v>info.jkprints@gmail.com</v>
       </c>
-      <c r="D35" s="1" t="str">
+      <c r="D35" t="str">
         <v/>
       </c>
-      <c r="E35" s="2">
+      <c r="E35">
         <v>170</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F35">
         <v>16.2</v>
       </c>
-      <c r="G35" s="4">
+      <c r="G35">
         <v>2.6</v>
       </c>
-      <c r="H35" s="5" t="d">
-        <v>2026-09-16T00:00:00.000Z</v>
+      <c r="H35" s="1" t="str">
+        <v>16/09/2026</v>
       </c>
     </row>
     <row r="36">
@@ -1291,20 +1277,20 @@
       <c r="C36" t="str">
         <v>JEREMY@JSA1BRANDEDCLOTHING.COM</v>
       </c>
-      <c r="D36" s="1" t="str">
+      <c r="D36" t="str">
         <v/>
       </c>
-      <c r="E36" s="2">
+      <c r="E36">
         <v>28</v>
       </c>
-      <c r="F36" s="3">
+      <c r="F36">
         <v>24.8</v>
       </c>
-      <c r="G36" s="4">
+      <c r="G36">
         <v>2.3</v>
       </c>
-      <c r="H36" s="5" t="d">
-        <v>2026-08-02T00:00:00.000Z</v>
+      <c r="H36" s="1" t="str">
+        <v>02/08/2026</v>
       </c>
     </row>
     <row r="37">
@@ -1317,20 +1303,20 @@
       <c r="C37" t="str">
         <v>info@wearejoeandco.co.uk</v>
       </c>
-      <c r="D37" s="1" t="str">
+      <c r="D37" t="str">
         <v/>
       </c>
-      <c r="E37" s="2">
+      <c r="E37">
         <v>62</v>
       </c>
-      <c r="F37" s="3">
+      <c r="F37">
         <v>23.3</v>
       </c>
-      <c r="G37" s="4">
+      <c r="G37">
         <v>1.87</v>
       </c>
-      <c r="H37" s="5" t="d">
-        <v>2026-04-16T00:00:00.000Z</v>
+      <c r="H37" s="1" t="str">
+        <v>16/04/2026</v>
       </c>
     </row>
     <row r="38">
@@ -1343,20 +1329,20 @@
       <c r="C38" t="str">
         <v>habib@keeps.london</v>
       </c>
-      <c r="D38" s="1" t="str">
+      <c r="D38" t="str">
         <v>07546821515</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38">
         <v>3</v>
       </c>
-      <c r="F38" s="3">
+      <c r="F38">
         <v>19</v>
       </c>
-      <c r="G38" s="4">
+      <c r="G38">
         <v>3.68</v>
       </c>
-      <c r="H38" s="5" t="d">
-        <v>2026-06-25T00:00:00.000Z</v>
+      <c r="H38" s="1" t="str">
+        <v>25/06/2026</v>
       </c>
     </row>
     <row r="39">
@@ -1369,10 +1355,10 @@
       <c r="C39" t="str">
         <v>sean@kit-room.co.uk</v>
       </c>
-      <c r="D39" s="1" t="str">
+      <c r="D39" t="str">
         <v/>
       </c>
-      <c r="E39" s="2">
+      <c r="E39">
         <v>0</v>
       </c>
     </row>
@@ -1386,20 +1372,20 @@
       <c r="C40" t="str">
         <v>accounts@kitco.biz</v>
       </c>
-      <c r="D40" s="1" t="str">
+      <c r="D40" t="str">
         <v>07737605765</v>
       </c>
-      <c r="E40" s="2">
+      <c r="E40">
         <v>23</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40">
         <v>69.1</v>
       </c>
-      <c r="G40" s="4">
+      <c r="G40">
         <v>1.75</v>
       </c>
-      <c r="H40" s="5" t="d">
-        <v>2026-09-10T00:00:00.000Z</v>
+      <c r="H40" s="1" t="str">
+        <v>10/09/2026</v>
       </c>
     </row>
     <row r="41">
@@ -1412,20 +1398,20 @@
       <c r="C41" t="str">
         <v>sales@klubcolours.com</v>
       </c>
-      <c r="D41" s="1" t="str">
+      <c r="D41" t="str">
         <v>07711500133</v>
       </c>
-      <c r="E41" s="2">
+      <c r="E41">
         <v>5</v>
       </c>
-      <c r="F41" s="3">
+      <c r="F41">
         <v>17.8</v>
       </c>
-      <c r="G41" s="4">
+      <c r="G41">
         <v>2.2</v>
       </c>
-      <c r="H41" s="5" t="d">
-        <v>2026-09-17T00:00:00.000Z</v>
+      <c r="H41" s="1" t="str">
+        <v>17/09/2026</v>
       </c>
     </row>
     <row r="42">
@@ -1438,20 +1424,20 @@
       <c r="C42" t="str">
         <v>kreativeembroidery@outlook.com</v>
       </c>
-      <c r="D42" s="1" t="str">
+      <c r="D42" t="str">
         <v>07917013100</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42">
         <v>7</v>
       </c>
-      <c r="F42" s="3">
+      <c r="F42">
         <v>105</v>
       </c>
-      <c r="G42" s="4">
+      <c r="G42">
         <v>3.02</v>
       </c>
-      <c r="H42" s="5" t="d">
-        <v>2026-05-25T00:00:00.000Z</v>
+      <c r="H42" s="1" t="str">
+        <v>25/05/2026</v>
       </c>
     </row>
     <row r="43">
@@ -1464,20 +1450,20 @@
       <c r="C43" t="str">
         <v>nick.clemente@logos-on.com</v>
       </c>
-      <c r="D43" s="1" t="str">
+      <c r="D43" t="str">
         <v/>
       </c>
-      <c r="E43" s="2">
+      <c r="E43">
         <v>255</v>
       </c>
-      <c r="F43" s="3">
+      <c r="F43">
         <v>15.9</v>
       </c>
-      <c r="G43" s="4">
+      <c r="G43">
         <v>2.13</v>
       </c>
-      <c r="H43" s="5" t="d">
-        <v>2026-09-01T00:00:00.000Z</v>
+      <c r="H43" s="1" t="str">
+        <v>01/09/2026</v>
       </c>
     </row>
     <row r="44">
@@ -1490,20 +1476,20 @@
       <c r="C44" t="str">
         <v>leicester@mdhteamwear.co.uk</v>
       </c>
-      <c r="D44" s="1" t="str">
+      <c r="D44" t="str">
         <v>01858 434812</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44">
         <v>16</v>
       </c>
-      <c r="F44" s="3">
+      <c r="F44">
         <v>50.2</v>
       </c>
-      <c r="G44" s="4">
+      <c r="G44">
         <v>1.57</v>
       </c>
-      <c r="H44" s="5" t="d">
-        <v>2026-08-31T00:00:00.000Z</v>
+      <c r="H44" s="1" t="str">
+        <v>31/08/2026</v>
       </c>
     </row>
     <row r="45">
@@ -1516,17 +1502,17 @@
       <c r="C45" t="str">
         <v>info@madforitmerch.co.uk</v>
       </c>
-      <c r="D45" s="1" t="str">
+      <c r="D45" t="str">
         <v/>
       </c>
-      <c r="E45" s="2">
+      <c r="E45">
         <v>11</v>
       </c>
-      <c r="F45" s="3">
+      <c r="F45">
         <v>4.5</v>
       </c>
-      <c r="H45" s="5" t="d">
-        <v>2025-12-12T00:00:00.000Z</v>
+      <c r="H45" s="1" t="str">
+        <v>12/12/2025</v>
       </c>
     </row>
     <row r="46">
@@ -1539,20 +1525,20 @@
       <c r="C46" t="str">
         <v>alastair@merch4.co.uk</v>
       </c>
-      <c r="D46" s="1" t="str">
+      <c r="D46" t="str">
         <v>07459 462 032</v>
       </c>
-      <c r="E46" s="2">
+      <c r="E46">
         <v>3</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46">
         <v>28.7</v>
       </c>
-      <c r="G46" s="4">
+      <c r="G46">
         <v>2.63</v>
       </c>
-      <c r="H46" s="5" t="d">
-        <v>2026-09-13T00:00:00.000Z</v>
+      <c r="H46" s="1" t="str">
+        <v>13/09/2026</v>
       </c>
     </row>
     <row r="47">
@@ -1565,20 +1551,20 @@
       <c r="C47" t="str">
         <v>sales@merox.co.uk</v>
       </c>
-      <c r="D47" s="1" t="str">
+      <c r="D47" t="str">
         <v>01202571210</v>
       </c>
-      <c r="E47" s="2">
+      <c r="E47">
         <v>2</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F47">
         <v>55</v>
       </c>
-      <c r="G47" s="4">
+      <c r="G47">
         <v>1.62</v>
       </c>
-      <c r="H47" s="5" t="d">
-        <v>2026-06-09T00:00:00.000Z</v>
+      <c r="H47" s="1" t="str">
+        <v>09/06/2026</v>
       </c>
     </row>
     <row r="48">
@@ -1591,10 +1577,10 @@
       <c r="C48" t="str">
         <v>mike@nativepromotions.com</v>
       </c>
-      <c r="D48" s="1" t="str">
+      <c r="D48" t="str">
         <v>01206 385 486</v>
       </c>
-      <c r="E48" s="2">
+      <c r="E48">
         <v>0</v>
       </c>
     </row>
@@ -1608,20 +1594,20 @@
       <c r="C49" t="str">
         <v>andy@needhamsuniforms.co.uk</v>
       </c>
-      <c r="D49" s="1" t="str">
+      <c r="D49" t="str">
         <v/>
       </c>
-      <c r="E49" s="2">
+      <c r="E49">
         <v>5</v>
       </c>
-      <c r="F49" s="3">
+      <c r="F49">
         <v>76.4</v>
       </c>
-      <c r="G49" s="4">
+      <c r="G49">
         <v>1.79</v>
       </c>
-      <c r="H49" s="5" t="d">
-        <v>2026-09-13T00:00:00.000Z</v>
+      <c r="H49" s="1" t="str">
+        <v>13/09/2026</v>
       </c>
     </row>
     <row r="50">
@@ -1634,20 +1620,20 @@
       <c r="C50" t="str">
         <v>peter@nextgenclothing.co.uk</v>
       </c>
-      <c r="D50" s="1" t="str">
+      <c r="D50" t="str">
         <v>07981 453392</v>
       </c>
-      <c r="E50" s="2">
+      <c r="E50">
         <v>11</v>
       </c>
-      <c r="F50" s="3">
+      <c r="F50">
         <v>392.4</v>
       </c>
-      <c r="G50" s="4">
+      <c r="G50">
         <v>1.45</v>
       </c>
-      <c r="H50" s="5" t="d">
-        <v>2026-07-19T00:00:00.000Z</v>
+      <c r="H50" s="1" t="str">
+        <v>19/07/2026</v>
       </c>
     </row>
     <row r="51">
@@ -1660,20 +1646,20 @@
       <c r="C51" t="str">
         <v>enquiries@oakhillembroidery.co.uk</v>
       </c>
-      <c r="D51" s="1" t="str">
+      <c r="D51" t="str">
         <v>07572458676</v>
       </c>
-      <c r="E51" s="2">
+      <c r="E51">
         <v>2</v>
       </c>
-      <c r="F51" s="3">
+      <c r="F51">
         <v>100</v>
       </c>
-      <c r="G51" s="4">
+      <c r="G51">
         <v>1.53</v>
       </c>
-      <c r="H51" s="5" t="d">
-        <v>2026-08-13T00:00:00.000Z</v>
+      <c r="H51" s="1" t="str">
+        <v>13/08/2026</v>
       </c>
     </row>
     <row r="52">
@@ -1686,20 +1672,20 @@
       <c r="C52" t="str">
         <v>sales@pcsports.co.uk</v>
       </c>
-      <c r="D52" s="1" t="str">
+      <c r="D52" t="str">
         <v/>
       </c>
-      <c r="E52" s="2">
+      <c r="E52">
         <v>163</v>
       </c>
-      <c r="F52" s="3">
+      <c r="F52">
         <v>57.4</v>
       </c>
-      <c r="G52" s="4">
+      <c r="G52">
         <v>1.7</v>
       </c>
-      <c r="H52" s="5" t="d">
-        <v>2026-09-14T00:00:00.000Z</v>
+      <c r="H52" s="1" t="str">
+        <v>14/09/2026</v>
       </c>
     </row>
     <row r="53">
@@ -1712,20 +1698,20 @@
       <c r="C53" t="str">
         <v>info@printmatterskent.com</v>
       </c>
-      <c r="D53" s="1" t="str">
+      <c r="D53" t="str">
         <v>01227 765031</v>
       </c>
-      <c r="E53" s="2">
+      <c r="E53">
         <v>4</v>
       </c>
-      <c r="F53" s="3">
+      <c r="F53">
         <v>292.8</v>
       </c>
-      <c r="G53" s="4">
+      <c r="G53">
         <v>1.66</v>
       </c>
-      <c r="H53" s="5" t="d">
-        <v>2026-07-30T00:00:00.000Z</v>
+      <c r="H53" s="1" t="str">
+        <v>30/07/2026</v>
       </c>
     </row>
     <row r="54">
@@ -1738,20 +1724,20 @@
       <c r="C54" t="str">
         <v>jono@positivebranding.co.uk</v>
       </c>
-      <c r="D54" s="1" t="str">
+      <c r="D54" t="str">
         <v>020 8912 1515</v>
       </c>
-      <c r="E54" s="2">
+      <c r="E54">
         <v>32</v>
       </c>
-      <c r="F54" s="3">
+      <c r="F54">
         <v>68.8</v>
       </c>
-      <c r="G54" s="4">
+      <c r="G54">
         <v>1.52</v>
       </c>
-      <c r="H54" s="5" t="d">
-        <v>2026-09-13T00:00:00.000Z</v>
+      <c r="H54" s="1" t="str">
+        <v>13/09/2026</v>
       </c>
     </row>
     <row r="55">
@@ -1764,17 +1750,17 @@
       <c r="C55" t="str">
         <v>nicolaraebrown@hotmail.com</v>
       </c>
-      <c r="D55" s="1" t="str">
+      <c r="D55" t="str">
         <v>07399834594</v>
       </c>
-      <c r="E55" s="2">
+      <c r="E55">
         <v>1</v>
       </c>
-      <c r="F55" s="3">
+      <c r="F55">
         <v>9</v>
       </c>
-      <c r="H55" s="5" t="d">
-        <v>2025-11-14T00:00:00.000Z</v>
+      <c r="H55" s="1" t="str">
+        <v>14/11/2025</v>
       </c>
     </row>
     <row r="56">
@@ -1787,10 +1773,10 @@
       <c r="C56" t="str">
         <v>clayton@protectivewearuk.com</v>
       </c>
-      <c r="D56" s="1" t="str">
+      <c r="D56" t="str">
         <v>01752 266374</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56">
         <v>0</v>
       </c>
     </row>
@@ -1804,20 +1790,20 @@
       <c r="C57" t="str">
         <v>info@purpleworkwear.co.uk</v>
       </c>
-      <c r="D57" s="1" t="str">
+      <c r="D57" t="str">
         <v/>
       </c>
-      <c r="E57" s="2">
+      <c r="E57">
         <v>157</v>
       </c>
-      <c r="F57" s="3">
+      <c r="F57">
         <v>15.1</v>
       </c>
-      <c r="G57" s="4">
+      <c r="G57">
         <v>2.29</v>
       </c>
-      <c r="H57" s="5" t="d">
-        <v>2026-09-18T00:00:00.000Z</v>
+      <c r="H57" s="1" t="str">
+        <v>18/09/2026</v>
       </c>
     </row>
     <row r="58">
@@ -1830,20 +1816,20 @@
       <c r="C58" t="str">
         <v>liam@redmonkeysigns.co.uk</v>
       </c>
-      <c r="D58" s="1" t="str">
+      <c r="D58" t="str">
         <v>01455 374325</v>
       </c>
-      <c r="E58" s="2">
+      <c r="E58">
         <v>1</v>
       </c>
-      <c r="F58" s="3">
+      <c r="F58">
         <v>240</v>
       </c>
-      <c r="G58" s="4">
+      <c r="G58">
         <v>1.74</v>
       </c>
-      <c r="H58" s="5" t="d">
-        <v>2026-09-03T00:00:00.000Z</v>
+      <c r="H58" s="1" t="str">
+        <v>03/09/2026</v>
       </c>
     </row>
     <row r="59">
@@ -1856,20 +1842,20 @@
       <c r="C59" t="str">
         <v>sales@relmsigns.co.uk</v>
       </c>
-      <c r="D59" s="1" t="str">
+      <c r="D59" t="str">
         <v>07966 275008</v>
       </c>
-      <c r="E59" s="2">
+      <c r="E59">
         <v>2</v>
       </c>
-      <c r="F59" s="3">
+      <c r="F59">
         <v>300</v>
       </c>
-      <c r="G59" s="4">
+      <c r="G59">
         <v>1.22</v>
       </c>
-      <c r="H59" s="5" t="d">
-        <v>2026-06-18T00:00:00.000Z</v>
+      <c r="H59" s="1" t="str">
+        <v>18/06/2026</v>
       </c>
     </row>
     <row r="60">
@@ -1882,20 +1868,20 @@
       <c r="C60" t="str">
         <v>sam@rutlandmerchandise.co.uk</v>
       </c>
-      <c r="D60" s="1" t="str">
+      <c r="D60" t="str">
         <v/>
       </c>
-      <c r="E60" s="2">
+      <c r="E60">
         <v>114</v>
       </c>
-      <c r="F60" s="3">
+      <c r="F60">
         <v>36.8</v>
       </c>
-      <c r="G60" s="4">
+      <c r="G60">
         <v>1.7</v>
       </c>
-      <c r="H60" s="5" t="d">
-        <v>2026-08-25T00:00:00.000Z</v>
+      <c r="H60" s="1" t="str">
+        <v>25/08/2026</v>
       </c>
     </row>
     <row r="61">
@@ -1908,20 +1894,20 @@
       <c r="C61" t="str">
         <v>accounts@shirtworks.co.uk</v>
       </c>
-      <c r="D61" s="1" t="str">
+      <c r="D61" t="str">
         <v/>
       </c>
-      <c r="E61" s="2">
+      <c r="E61">
         <v>138</v>
       </c>
-      <c r="F61" s="3">
+      <c r="F61">
         <v>23.7</v>
       </c>
-      <c r="G61" s="4">
+      <c r="G61">
         <v>1.77</v>
       </c>
-      <c r="H61" s="5" t="d">
-        <v>2026-09-17T00:00:00.000Z</v>
+      <c r="H61" s="1" t="str">
+        <v>17/09/2026</v>
       </c>
     </row>
     <row r="62">
@@ -1934,20 +1920,20 @@
       <c r="C62" t="str">
         <v>safetycentre@hotmail.co.uk</v>
       </c>
-      <c r="D62" s="1" t="str">
+      <c r="D62" t="str">
         <v>02083958913</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62">
         <v>5</v>
       </c>
-      <c r="F62" s="3">
+      <c r="F62">
         <v>58.4</v>
       </c>
-      <c r="G62" s="4">
+      <c r="G62">
         <v>1.72</v>
       </c>
-      <c r="H62" s="5" t="d">
-        <v>2026-08-31T00:00:00.000Z</v>
+      <c r="H62" s="1" t="str">
+        <v>31/08/2026</v>
       </c>
     </row>
     <row r="63">
@@ -1960,20 +1946,20 @@
       <c r="C63" t="str">
         <v>info@surreysports.shop</v>
       </c>
-      <c r="D63" s="1" t="str">
+      <c r="D63" t="str">
         <v>01737 881211</v>
       </c>
-      <c r="E63" s="2">
+      <c r="E63">
         <v>6</v>
       </c>
-      <c r="F63" s="3">
+      <c r="F63">
         <v>28.5</v>
       </c>
-      <c r="G63" s="4">
+      <c r="G63">
         <v>2.3</v>
       </c>
-      <c r="H63" s="5" t="d">
-        <v>2026-06-09T00:00:00.000Z</v>
+      <c r="H63" s="1" t="str">
+        <v>09/06/2026</v>
       </c>
     </row>
     <row r="64">
@@ -1986,20 +1972,20 @@
       <c r="C64" t="str">
         <v>info@toasports.co.uk</v>
       </c>
-      <c r="D64" s="1" t="str">
+      <c r="D64" t="str">
         <v>07714755182</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64">
         <v>34</v>
       </c>
-      <c r="F64" s="3">
+      <c r="F64">
         <v>12.3</v>
       </c>
-      <c r="G64" s="4">
+      <c r="G64">
         <v>2.26</v>
       </c>
-      <c r="H64" s="5" t="d">
-        <v>2026-09-14T00:00:00.000Z</v>
+      <c r="H64" s="1" t="str">
+        <v>14/09/2026</v>
       </c>
     </row>
     <row r="65">
@@ -2012,20 +1998,20 @@
       <c r="C65" t="str">
         <v>stuartmcadie@gmail.com</v>
       </c>
-      <c r="D65" s="1" t="str">
+      <c r="D65" t="str">
         <v>07970 494424</v>
       </c>
-      <c r="E65" s="2">
+      <c r="E65">
         <v>28</v>
       </c>
-      <c r="F65" s="3">
+      <c r="F65">
         <v>14</v>
       </c>
-      <c r="G65" s="4">
+      <c r="G65">
         <v>1.69</v>
       </c>
-      <c r="H65" s="5" t="d">
-        <v>2026-09-08T00:00:00.000Z</v>
+      <c r="H65" s="1" t="str">
+        <v>08/09/2026</v>
       </c>
     </row>
     <row r="66">
@@ -2038,20 +2024,20 @@
       <c r="C66" t="str">
         <v>sales@beelineonline.co.uk</v>
       </c>
-      <c r="D66" s="1" t="str">
+      <c r="D66" t="str">
         <v>07737 216963</v>
       </c>
-      <c r="E66" s="2">
+      <c r="E66">
         <v>2</v>
       </c>
-      <c r="F66" s="3">
+      <c r="F66">
         <v>19</v>
       </c>
-      <c r="G66" s="4">
+      <c r="G66">
         <v>2.04</v>
       </c>
-      <c r="H66" s="5" t="d">
-        <v>2026-04-14T00:00:00.000Z</v>
+      <c r="H66" s="1" t="str">
+        <v>14/04/2026</v>
       </c>
     </row>
     <row r="67">
@@ -2064,10 +2050,10 @@
       <c r="C67" t="str">
         <v>info@theliverpool.shop</v>
       </c>
-      <c r="D67" s="1" t="str">
+      <c r="D67" t="str">
         <v>07824600735</v>
       </c>
-      <c r="E67" s="2">
+      <c r="E67">
         <v>0</v>
       </c>
     </row>
@@ -2081,20 +2067,20 @@
       <c r="C68" t="str">
         <v>THELOGOFARM@OUTLOOK.COM</v>
       </c>
-      <c r="D68" s="1" t="str">
+      <c r="D68" t="str">
         <v>07895 963050</v>
       </c>
-      <c r="E68" s="2">
+      <c r="E68">
         <v>29</v>
       </c>
-      <c r="F68" s="3">
+      <c r="F68">
         <v>113.4</v>
       </c>
-      <c r="G68" s="4">
+      <c r="G68">
         <v>1.55</v>
       </c>
-      <c r="H68" s="5" t="d">
-        <v>2026-08-16T00:00:00.000Z</v>
+      <c r="H68" s="1" t="str">
+        <v>16/08/2026</v>
       </c>
     </row>
     <row r="69">
@@ -2107,10 +2093,10 @@
       <c r="C69" t="str">
         <v>theyorkshirebrand@outlook.com</v>
       </c>
-      <c r="D69" s="1" t="str">
+      <c r="D69" t="str">
         <v>07543 157132</v>
       </c>
-      <c r="E69" s="2">
+      <c r="E69">
         <v>0</v>
       </c>
     </row>
@@ -2124,20 +2110,20 @@
       <c r="C70" t="str">
         <v>paulramsden@tg24.com</v>
       </c>
-      <c r="D70" s="1" t="str">
+      <c r="D70" t="str">
         <v>+447767252639</v>
       </c>
-      <c r="E70" s="2">
+      <c r="E70">
         <v>1</v>
       </c>
-      <c r="F70" s="3">
+      <c r="F70">
         <v>106</v>
       </c>
-      <c r="G70" s="4">
+      <c r="G70">
         <v>1.52</v>
       </c>
-      <c r="H70" s="5" t="d">
-        <v>2026-06-25T00:00:00.000Z</v>
+      <c r="H70" s="1" t="str">
+        <v>25/06/2026</v>
       </c>
     </row>
     <row r="71">
@@ -2150,20 +2136,20 @@
       <c r="C71" t="str">
         <v>rob@treblethree.co.uk</v>
       </c>
-      <c r="D71" s="1" t="str">
+      <c r="D71" t="str">
         <v>01524 8051114</v>
       </c>
-      <c r="E71" s="2">
+      <c r="E71">
         <v>31</v>
       </c>
-      <c r="F71" s="3">
+      <c r="F71">
         <v>4.2</v>
       </c>
-      <c r="G71" s="4">
+      <c r="G71">
         <v>2.36</v>
       </c>
-      <c r="H71" s="5" t="d">
-        <v>2026-03-06T00:00:00.000Z</v>
+      <c r="H71" s="1" t="str">
+        <v>06/03/2026</v>
       </c>
     </row>
     <row r="72">
@@ -2176,20 +2162,20 @@
       <c r="C72" t="str">
         <v>turnbullsfc@yahoo.com</v>
       </c>
-      <c r="D72" s="1" t="str">
+      <c r="D72" t="str">
         <v>07518196469</v>
       </c>
-      <c r="E72" s="2">
+      <c r="E72">
         <v>7</v>
       </c>
-      <c r="F72" s="3">
+      <c r="F72">
         <v>32.4</v>
       </c>
-      <c r="G72" s="4">
+      <c r="G72">
         <v>2.55</v>
       </c>
-      <c r="H72" s="5" t="d">
-        <v>2026-07-08T00:00:00.000Z</v>
+      <c r="H72" s="1" t="str">
+        <v>08/07/2026</v>
       </c>
     </row>
     <row r="73">
@@ -2202,20 +2188,20 @@
       <c r="C73" t="str">
         <v>info@twentytwoshop.com</v>
       </c>
-      <c r="D73" s="1" t="str">
+      <c r="D73" t="str">
         <v/>
       </c>
-      <c r="E73" s="2">
+      <c r="E73">
         <v>7</v>
       </c>
-      <c r="F73" s="3">
+      <c r="F73">
         <v>55.3</v>
       </c>
-      <c r="G73" s="4">
+      <c r="G73">
         <v>2.42</v>
       </c>
-      <c r="H73" s="5" t="d">
-        <v>2026-05-17T00:00:00.000Z</v>
+      <c r="H73" s="1" t="str">
+        <v>17/05/2026</v>
       </c>
     </row>
     <row r="74">
@@ -2228,10 +2214,10 @@
       <c r="C74" t="str">
         <v>raj@uk-infinity.com</v>
       </c>
-      <c r="D74" s="1" t="str">
+      <c r="D74" t="str">
         <v>07855 665515</v>
       </c>
-      <c r="E74" s="2">
+      <c r="E74">
         <v>0</v>
       </c>
     </row>
@@ -2245,20 +2231,20 @@
       <c r="C75" t="str">
         <v>info@wearunifab.com</v>
       </c>
-      <c r="D75" s="1" t="str">
+      <c r="D75" t="str">
         <v/>
       </c>
-      <c r="E75" s="2">
+      <c r="E75">
         <v>3</v>
       </c>
-      <c r="F75" s="3">
+      <c r="F75">
         <v>26</v>
       </c>
-      <c r="G75" s="4">
+      <c r="G75">
         <v>2.34</v>
       </c>
-      <c r="H75" s="5" t="d">
-        <v>2026-09-14T00:00:00.000Z</v>
+      <c r="H75" s="1" t="str">
+        <v>14/09/2026</v>
       </c>
     </row>
     <row r="76">
@@ -2271,20 +2257,20 @@
       <c r="C76" t="str">
         <v>cland@uniformsforwork.com</v>
       </c>
-      <c r="D76" s="1" t="str">
+      <c r="D76" t="str">
         <v>+447899904151</v>
       </c>
-      <c r="E76" s="2">
+      <c r="E76">
         <v>8</v>
       </c>
-      <c r="F76" s="3">
+      <c r="F76">
         <v>163.3</v>
       </c>
-      <c r="G76" s="4">
+      <c r="G76">
         <v>1.42</v>
       </c>
-      <c r="H76" s="5" t="d">
-        <v>2026-09-10T00:00:00.000Z</v>
+      <c r="H76" s="1" t="str">
+        <v>10/09/2026</v>
       </c>
     </row>
     <row r="77">
@@ -2297,20 +2283,20 @@
       <c r="C77" t="str">
         <v>vanessa@universaluniform.co.uk</v>
       </c>
-      <c r="D77" s="1" t="str">
+      <c r="D77" t="str">
         <v>01242580062</v>
       </c>
-      <c r="E77" s="2">
+      <c r="E77">
         <v>21</v>
       </c>
-      <c r="F77" s="3">
+      <c r="F77">
         <v>27.7</v>
       </c>
-      <c r="G77" s="4">
+      <c r="G77">
         <v>1.81</v>
       </c>
-      <c r="H77" s="5" t="d">
-        <v>2026-09-18T00:00:00.000Z</v>
+      <c r="H77" s="1" t="str">
+        <v>18/09/2026</v>
       </c>
     </row>
     <row r="78">
@@ -2323,17 +2309,17 @@
       <c r="C78" t="str">
         <v>phil@vx-3.com</v>
       </c>
-      <c r="D78" s="1" t="str">
+      <c r="D78" t="str">
         <v>01803 524623</v>
       </c>
-      <c r="E78" s="2">
+      <c r="E78">
         <v>46</v>
       </c>
-      <c r="F78" s="3">
+      <c r="F78">
         <v>59.6</v>
       </c>
-      <c r="H78" s="5" t="d">
-        <v>2025-12-15T00:00:00.000Z</v>
+      <c r="H78" s="1" t="str">
+        <v>15/12/2025</v>
       </c>
     </row>
     <row r="79">
@@ -2346,20 +2332,20 @@
       <c r="C79" t="str">
         <v>hello@vibrantcolour.co.uk</v>
       </c>
-      <c r="D79" s="1" t="str">
+      <c r="D79" t="str">
         <v>01733 736936</v>
       </c>
-      <c r="E79" s="2">
+      <c r="E79">
         <v>33</v>
       </c>
-      <c r="F79" s="3">
+      <c r="F79">
         <v>90.6</v>
       </c>
-      <c r="G79" s="4">
+      <c r="G79">
         <v>1.79</v>
       </c>
-      <c r="H79" s="5" t="d">
-        <v>2026-09-08T00:00:00.000Z</v>
+      <c r="H79" s="1" t="str">
+        <v>08/09/2026</v>
       </c>
     </row>
     <row r="80">
@@ -2372,20 +2358,20 @@
       <c r="C80" t="str">
         <v>darren@wcsscotland.com</v>
       </c>
-      <c r="D80" s="1" t="str">
+      <c r="D80" t="str">
         <v/>
       </c>
-      <c r="E80" s="2">
+      <c r="E80">
         <v>5</v>
       </c>
-      <c r="F80" s="3">
+      <c r="F80">
         <v>133</v>
       </c>
-      <c r="G80" s="4">
+      <c r="G80">
         <v>1.46</v>
       </c>
-      <c r="H80" s="5" t="d">
-        <v>2026-08-04T00:00:00.000Z</v>
+      <c r="H80" s="1" t="str">
+        <v>04/08/2026</v>
       </c>
     </row>
     <row r="81">
@@ -2398,20 +2384,20 @@
       <c r="C81" t="str">
         <v>TASMINPERRIER@HOTMAIL.COM</v>
       </c>
-      <c r="D81" s="1" t="str">
+      <c r="D81" t="str">
         <v/>
       </c>
-      <c r="E81" s="2">
+      <c r="E81">
         <v>6</v>
       </c>
-      <c r="F81" s="3">
+      <c r="F81">
         <v>5</v>
       </c>
-      <c r="G81" s="4">
+      <c r="G81">
         <v>6.16</v>
       </c>
-      <c r="H81" s="5" t="d">
-        <v>2026-03-27T00:00:00.000Z</v>
+      <c r="H81" s="1" t="str">
+        <v>27/03/2026</v>
       </c>
     </row>
     <row r="82">
@@ -2424,10 +2410,10 @@
       <c r="C82" t="str">
         <v>matt@mantisworld.com</v>
       </c>
-      <c r="D82" s="1" t="str">
+      <c r="D82" t="str">
         <v/>
       </c>
-      <c r="E82" s="2">
+      <c r="E82">
         <v>0</v>
       </c>
     </row>

</xml_diff>